<commit_message>
Add email reference (143952-0-0-00-FRP) column to HS summary
Both packages share the same reference, so the reference division
coincides with the P35/Q35 package split; noted in the file.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P7dj9YaDaJdQUHninPzxpV
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Hitachi_143952.xlsx
+++ b/output/HS_Code_Summary_Hitachi_143952.xlsx
@@ -491,20 +491,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="6" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="38" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -517,7 +518,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Odesílatel (oba balíčky): Hitachi Energy Czech Republic s.r.o., Průmyslová 137, 541 01 Trutnov | Příjemce: Wijnne Barends Logistics B.V., Eemshaven, NL | 2 balíčky = 2 VDD (P35, Q35) | Objednávka: 4501839901 | Reference: 143952-0-0-00-FRP</t>
+          <t>Odesílatel (oba balíčky): Hitachi Energy Czech Republic s.r.o., Průmyslová 137, 541 01 Trutnov | Příjemce: Wijnne Barends Logistics B.V., Eemshaven, NL | 2 balíčky = 2 VDD (P35, Q35) | Objednávka: 4501839901</t>
         </is>
       </c>
     </row>
@@ -529,50 +530,55 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
+          <t>Reference (e-mail)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
           <t>HS kód</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Popis (CZ)</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Země původu</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Množství</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>MJ</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Čistá hmotnost (kg)</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Hrubá hmotnost (kg)</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Celní hodnota (EUR)</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>CBAM</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>Antidumping</t>
         </is>
@@ -586,38 +592,43 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
+          <t>143952-0-0-00-FRP</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
           <t>73269098</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>Ostatní výrobky ze železa nebo oceli, které nejsou nikde jinde specifikovány</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>CZ</t>
         </is>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="F5" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="G5" s="4" t="n"/>
       <c r="H5" s="4" t="n"/>
-      <c r="I5" s="6" t="n">
+      <c r="I5" s="4" t="n"/>
+      <c r="J5" s="6" t="n">
         <v>10.89</v>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>Ano (příloha I CBAM)</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr"/>
+      <c r="L5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -627,38 +638,43 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
+          <t>143952-0-0-00-FRP</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
           <t>73181650</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Samosvorné matice</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="F6" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="G6" s="4" t="n"/>
       <c r="H6" s="4" t="n"/>
-      <c r="I6" s="6" t="n">
+      <c r="I6" s="4" t="n"/>
+      <c r="J6" s="6" t="n">
         <v>0.52</v>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="K6" s="4" t="inlineStr">
         <is>
           <t>Ano (příloha I CBAM)</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="L6" s="5" t="inlineStr">
         <is>
           <t>Spojovací materiál ze železa/oceli původem CN — dovoz do EU podléhá antidumpingu (nař. 2022/191)</t>
         </is>
@@ -672,38 +688,43 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
+          <t>143952-0-0-00-FRP</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
           <t>74153300</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Šrouby, vruty, svorníky (maticové šrouby) a matice z mědi, případně ze železa nebo oceli s měděnou hlavou</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="F7" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="G7" s="4" t="n"/>
       <c r="H7" s="4" t="n"/>
-      <c r="I7" s="6" t="n">
+      <c r="I7" s="4" t="n"/>
+      <c r="J7" s="6" t="n">
         <v>0.35</v>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="K7" s="4" t="inlineStr">
         <is>
           <t>Ne</t>
         </is>
       </c>
-      <c r="K7" s="5" t="inlineStr"/>
+      <c r="L7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -713,38 +734,43 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
+          <t>143952-0-0-00-FRP</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
           <t>39269097</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Ostatní výrobky z plastů, které nejsou jinde specifikovány</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>CZ</t>
         </is>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="F8" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="G8" s="4" t="n"/>
       <c r="H8" s="4" t="n"/>
-      <c r="I8" s="6" t="n">
+      <c r="I8" s="4" t="n"/>
+      <c r="J8" s="6" t="n">
         <v>1002.9</v>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="K8" s="4" t="inlineStr">
         <is>
           <t>Ne</t>
         </is>
       </c>
-      <c r="K8" s="5" t="inlineStr"/>
+      <c r="L8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -754,38 +780,43 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
+          <t>143952-0-0-00-FRP</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
           <t>85381000</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>Tabule, panely, ovládací stoly, pulty, skříně a jiné základny pro elektrické řízení nebo rozvod elektřiny, které nejsou vybaveny příslušnými přístroji</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>CZ</t>
         </is>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="F9" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="G9" s="4" t="n"/>
       <c r="H9" s="4" t="n"/>
-      <c r="I9" s="6" t="n">
+      <c r="I9" s="4" t="n"/>
+      <c r="J9" s="6" t="n">
         <v>32.87</v>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="K9" s="4" t="inlineStr">
         <is>
           <t>Ne</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr"/>
+      <c r="L9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -795,38 +826,43 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
+          <t>143952-0-0-00-FRP</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
           <t>40169300</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>Plochá těsnění, podložky a jiná těsnění</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>AT</t>
         </is>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="F10" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="G10" s="4" t="n"/>
       <c r="H10" s="4" t="n"/>
-      <c r="I10" s="6" t="n">
+      <c r="I10" s="4" t="n"/>
+      <c r="J10" s="6" t="n">
         <v>1.9</v>
       </c>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="K10" s="4" t="inlineStr">
         <is>
           <t>Ne</t>
         </is>
       </c>
-      <c r="K10" s="5" t="inlineStr"/>
+      <c r="L10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -834,26 +870,31 @@
           <t>P35 celkem (faktura 810678973)</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n"/>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>143952-0-0-00-FRP</t>
+        </is>
+      </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7">
-        <f>SUM(E5:E10)</f>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="7">
+        <f>SUM(F5:F10)</f>
         <v>37</v>
       </c>
-      <c r="F11" s="7" t="n"/>
-      <c r="G11" s="8" t="n">
+      <c r="G11" s="7" t="n"/>
+      <c r="H11" s="8" t="n">
         <v>2.5</v>
       </c>
-      <c r="H11" s="8" t="n">
+      <c r="I11" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="I11" s="9">
-        <f>SUM(I5:I10)</f>
+      <c r="J11" s="9">
+        <f>SUM(J5:J10)</f>
         <v>1049.43</v>
       </c>
-      <c r="J11" s="7" t="n"/>
       <c r="K11" s="7" t="n"/>
+      <c r="L11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -863,38 +904,43 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
+          <t>143952-0-0-00-FRP</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
           <t>85381000</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>Tabule, panely, ovládací stoly, pulty, skříně a jiné základny pro elektrické řízení nebo rozvod elektřiny, které nejsou vybaveny příslušnými přístroji</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>CZ</t>
         </is>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="F12" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="G12" s="4" t="n"/>
       <c r="H12" s="4" t="n"/>
-      <c r="I12" s="6" t="n">
+      <c r="I12" s="4" t="n"/>
+      <c r="J12" s="6" t="n">
         <v>53.66</v>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="K12" s="4" t="inlineStr">
         <is>
           <t>Ne</t>
         </is>
       </c>
-      <c r="K12" s="5" t="inlineStr"/>
+      <c r="L12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -904,38 +950,43 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
+          <t>143952-0-0-00-FRP</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
           <t>74153300</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>Šrouby, vruty, svorníky (maticové šrouby) a matice z mědi, případně ze železa nebo oceli s měděnou hlavou</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="F13" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="G13" s="4" t="n"/>
       <c r="H13" s="4" t="n"/>
-      <c r="I13" s="6" t="n">
+      <c r="I13" s="4" t="n"/>
+      <c r="J13" s="6" t="n">
         <v>0.64</v>
       </c>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="K13" s="4" t="inlineStr">
         <is>
           <t>Ne</t>
         </is>
       </c>
-      <c r="K13" s="5" t="inlineStr"/>
+      <c r="L13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -945,38 +996,43 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
+          <t>143952-0-0-00-FRP</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
           <t>40169300</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>Plochá těsnění, podložky a jiná těsnění</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>AT</t>
         </is>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="F14" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="G14" s="4" t="n"/>
       <c r="H14" s="4" t="n"/>
-      <c r="I14" s="6" t="n">
+      <c r="I14" s="4" t="n"/>
+      <c r="J14" s="6" t="n">
         <v>1.9</v>
       </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="K14" s="4" t="inlineStr">
         <is>
           <t>Ne</t>
         </is>
       </c>
-      <c r="K14" s="5" t="inlineStr"/>
+      <c r="L14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -986,38 +1042,43 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
+          <t>143952-0-0-00-FRP</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
           <t>73181650</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>Samosvorné matice</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="F15" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="G15" s="4" t="n"/>
       <c r="H15" s="4" t="n"/>
-      <c r="I15" s="6" t="n">
+      <c r="I15" s="4" t="n"/>
+      <c r="J15" s="6" t="n">
         <v>0.08</v>
       </c>
-      <c r="J15" s="4" t="inlineStr">
+      <c r="K15" s="4" t="inlineStr">
         <is>
           <t>Ano (příloha I CBAM)</t>
         </is>
       </c>
-      <c r="K15" s="5" t="inlineStr">
+      <c r="L15" s="5" t="inlineStr">
         <is>
           <t>Spojovací materiál ze železa/oceli původem CN — dovoz do EU podléhá antidumpingu (nař. 2022/191)</t>
         </is>
@@ -1029,26 +1090,31 @@
           <t>Q35 celkem (faktura 810678974)</t>
         </is>
       </c>
-      <c r="B16" s="7" t="n"/>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>143952-0-0-00-FRP</t>
+        </is>
+      </c>
       <c r="C16" s="7" t="n"/>
       <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7">
-        <f>SUM(E12:E15)</f>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7">
+        <f>SUM(F12:F15)</f>
         <v>34</v>
       </c>
-      <c r="F16" s="7" t="n"/>
-      <c r="G16" s="8" t="n">
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="8" t="n">
         <v>1.5</v>
       </c>
-      <c r="H16" s="8" t="n">
+      <c r="I16" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="I16" s="9">
-        <f>SUM(I12:I15)</f>
+      <c r="J16" s="9">
+        <f>SUM(J12:J15)</f>
         <v>56.28</v>
       </c>
-      <c r="J16" s="7" t="n"/>
       <c r="K16" s="7" t="n"/>
+      <c r="L16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
@@ -1061,20 +1127,21 @@
       <c r="D17" s="10" t="n"/>
       <c r="E17" s="10" t="n"/>
       <c r="F17" s="10" t="n"/>
-      <c r="G17" s="11">
-        <f>G11+G16</f>
-        <v>4</v>
-      </c>
+      <c r="G17" s="10" t="n"/>
       <c r="H17" s="11">
         <f>H11+H16</f>
+        <v>4</v>
+      </c>
+      <c r="I17" s="11">
+        <f>I11+I16</f>
         <v>5</v>
       </c>
-      <c r="I17" s="12">
-        <f>I11+I16</f>
+      <c r="J17" s="12">
+        <f>J11+J16</f>
         <v>1105.71</v>
       </c>
-      <c r="J17" s="10" t="n"/>
       <c r="K17" s="10" t="n"/>
+      <c r="L17" s="10" t="n"/>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="13" t="inlineStr">
@@ -1084,72 +1151,80 @@
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="14" t="inlineStr">
-        <is>
-          <t>⚠ PREFERENČNÍ VĚTA: V dokladech (faktury 810678973/810678974, dodací listy) NENÍ uvedena žádná preferenční věta o původu. Zboží nemá deklarován preferenční původ.</t>
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>• REFERENCE: Oba balíčky (P35 i Q35) mají v e-mailu STEJNOU referenci 143952-0-0-00-FRP — dělení podle reference se tedy kryje s dělením podle balíčků. Číslo objednávky 4501839901 (pro interní účtování Hitachi) je uvedeno v hlavičce.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="14" t="inlineStr">
         <is>
+          <t>⚠ PREFERENČNÍ VĚTA: V dokladech (faktury 810678973/810678974, dodací listy) NENÍ uvedena žádná preferenční věta o původu. Zboží nemá deklarován preferenční původ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
           <t>⚠ HMOTNOSTI: Faktury uvádějí u všech položek 'Net Weight 0' — čistá/hrubá hmotnost na úrovni jednotlivých HS kódů NENÍ v podkladech k dispozici. Uvedeny jsou pouze hmotnosti za balíček (P35: NW 2,5 kg / GW 3 kg; Q35: NW 1,5 kg / GW 2 kg — zdroj: e-mail Hitachi + dodací listy). Sloupce ponechány dle pravidel.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="15" t="inlineStr">
-        <is>
-          <t>• Hodnoty řádků odpovídají fakturám: P35 = 1 049,43 EUR (faktura 810678973), Q35 = 56,28 EUR (faktura 810678974). Kontrolní součty sedí na fakturované částky.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>• CBAM: kódy 7318/7326 (železo/ocel) jsou v příloze I nařízení CBAM — relevantní při dovozu do EU; tato zásilka je vývoz z EU, CBAM se na ni tedy přímo nevztahuje.</t>
+          <t>• Hodnoty řádků odpovídají fakturám: P35 = 1 049,43 EUR (faktura 810678973), Q35 = 56,28 EUR (faktura 810678974). Kontrolní součty sedí na fakturované částky.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
+          <t>• CBAM: kódy 7318/7326 (železo/ocel) jsou v příloze I nařízení CBAM — relevantní při dovozu do EU; tato zásilka je vývoz z EU, CBAM se na ni tedy přímo nevztahuje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="15" t="inlineStr">
+        <is>
           <t>• Antidumping: samosvorné matice (73181650) původem z Číny podléhají při dovozu do EU antidumpingovému clu na spojovací materiál (nař. 2022/191) — pro tento vývoz bez přímého dopadu, uvedeno pro úplnost.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="15" customHeight="1">
-      <c r="A25" s="15" t="inlineStr">
-        <is>
-          <t>• Popisy (CZ) dodány zákazníkem e-mailem (Iva Kolertová, Hitachi Energy, 20.07.2026).</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>• Bez obchodní slevy — žádná sleva na fakturách uvedena není.</t>
+          <t>• Popisy (CZ) dodány zákazníkem e-mailem (Iva Kolertová, Hitachi Energy, 20.07.2026).</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="15" t="inlineStr">
         <is>
+          <t>• Bez obchodní slevy — žádná sleva na fakturách uvedena není.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="15" customHeight="1">
+      <c r="A28" s="15" t="inlineStr">
+        <is>
           <t>• Incoterm CPT Eemshaven (dle pravidel neuveden jako sloupec). Projekt: offshore Nordsee 2 / Godewind.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A22:K22"/>
-    <mergeCell ref="A20:K20"/>
-    <mergeCell ref="A21:K21"/>
-    <mergeCell ref="A26:K26"/>
-    <mergeCell ref="A25:K25"/>
-    <mergeCell ref="A24:K24"/>
-    <mergeCell ref="A19:K19"/>
-    <mergeCell ref="A23:K23"/>
-    <mergeCell ref="A27:K27"/>
+  <mergeCells count="10">
+    <mergeCell ref="A20:L20"/>
+    <mergeCell ref="A24:L24"/>
+    <mergeCell ref="A26:L26"/>
+    <mergeCell ref="A25:L25"/>
+    <mergeCell ref="A19:L19"/>
+    <mergeCell ref="A28:L28"/>
+    <mergeCell ref="A23:L23"/>
+    <mergeCell ref="A22:L22"/>
+    <mergeCell ref="A27:L27"/>
+    <mergeCell ref="A21:L21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add estimated net weights per HS code
Per-line weights are absent from the invoices (Net Weight 0), so net
weights are allocated approximately by item type and scaled to match
the documented package totals (P35: 2.5 kg, Q35: 1.5 kg). Estimates
are italicized and flagged in the notes.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P7dj9YaDaJdQUHninPzxpV
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Hitachi_143952.xlsx
+++ b/output/HS_Code_Summary_Hitachi_143952.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,6 +44,10 @@
     </font>
     <font>
       <name val="Arial"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -99,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -110,17 +114,20 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -491,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -501,7 +508,7 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
@@ -560,7 +567,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Čistá hmotnost (kg)</t>
+          <t>Čistá hmotnost (kg) — ODHAD</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -618,9 +625,11 @@
           <t>PC</t>
         </is>
       </c>
-      <c r="H5" s="4" t="n"/>
+      <c r="H5" s="6" t="n">
+        <v>0.5</v>
+      </c>
       <c r="I5" s="4" t="n"/>
-      <c r="J5" s="6" t="n">
+      <c r="J5" s="7" t="n">
         <v>10.89</v>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -664,9 +673,11 @@
           <t>PC</t>
         </is>
       </c>
-      <c r="H6" s="4" t="n"/>
+      <c r="H6" s="6" t="n">
+        <v>0.02</v>
+      </c>
       <c r="I6" s="4" t="n"/>
-      <c r="J6" s="6" t="n">
+      <c r="J6" s="7" t="n">
         <v>0.52</v>
       </c>
       <c r="K6" s="4" t="inlineStr">
@@ -714,9 +725,11 @@
           <t>PC</t>
         </is>
       </c>
-      <c r="H7" s="4" t="n"/>
+      <c r="H7" s="6" t="n">
+        <v>0.03</v>
+      </c>
       <c r="I7" s="4" t="n"/>
-      <c r="J7" s="6" t="n">
+      <c r="J7" s="7" t="n">
         <v>0.35</v>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -760,9 +773,11 @@
           <t>PC</t>
         </is>
       </c>
-      <c r="H8" s="4" t="n"/>
+      <c r="H8" s="6" t="n">
+        <v>1.8</v>
+      </c>
       <c r="I8" s="4" t="n"/>
-      <c r="J8" s="6" t="n">
+      <c r="J8" s="7" t="n">
         <v>1002.9</v>
       </c>
       <c r="K8" s="4" t="inlineStr">
@@ -806,9 +821,11 @@
           <t>PC</t>
         </is>
       </c>
-      <c r="H9" s="4" t="n"/>
+      <c r="H9" s="6" t="n">
+        <v>0.1</v>
+      </c>
       <c r="I9" s="4" t="n"/>
-      <c r="J9" s="6" t="n">
+      <c r="J9" s="7" t="n">
         <v>32.87</v>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -852,9 +869,11 @@
           <t>M</t>
         </is>
       </c>
-      <c r="H10" s="4" t="n"/>
+      <c r="H10" s="6" t="n">
+        <v>0.05</v>
+      </c>
       <c r="I10" s="4" t="n"/>
-      <c r="J10" s="6" t="n">
+      <c r="J10" s="7" t="n">
         <v>1.9</v>
       </c>
       <c r="K10" s="4" t="inlineStr">
@@ -865,36 +884,37 @@
       <c r="L10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>P35 celkem (faktura 810678973)</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>143952-0-0-00-FRP</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
-      <c r="F11" s="7">
+      <c r="C11" s="8" t="n"/>
+      <c r="D11" s="8" t="n"/>
+      <c r="E11" s="8" t="n"/>
+      <c r="F11" s="8">
         <f>SUM(F5:F10)</f>
         <v>37</v>
       </c>
-      <c r="G11" s="7" t="n"/>
-      <c r="H11" s="8" t="n">
+      <c r="G11" s="8" t="n"/>
+      <c r="H11" s="9">
+        <f>SUM(H5:H10)</f>
         <v>2.5</v>
       </c>
-      <c r="I11" s="8" t="n">
+      <c r="I11" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="J11" s="9">
+      <c r="J11" s="11">
         <f>SUM(J5:J10)</f>
         <v>1049.43</v>
       </c>
-      <c r="K11" s="7" t="n"/>
-      <c r="L11" s="7" t="n"/>
+      <c r="K11" s="8" t="n"/>
+      <c r="L11" s="8" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -930,9 +950,11 @@
           <t>PC</t>
         </is>
       </c>
-      <c r="H12" s="4" t="n"/>
+      <c r="H12" s="6" t="n">
+        <v>1.4</v>
+      </c>
       <c r="I12" s="4" t="n"/>
-      <c r="J12" s="6" t="n">
+      <c r="J12" s="7" t="n">
         <v>53.66</v>
       </c>
       <c r="K12" s="4" t="inlineStr">
@@ -976,9 +998,11 @@
           <t>PC</t>
         </is>
       </c>
-      <c r="H13" s="4" t="n"/>
+      <c r="H13" s="6" t="n">
+        <v>0.04</v>
+      </c>
       <c r="I13" s="4" t="n"/>
-      <c r="J13" s="6" t="n">
+      <c r="J13" s="7" t="n">
         <v>0.64</v>
       </c>
       <c r="K13" s="4" t="inlineStr">
@@ -1022,9 +1046,11 @@
           <t>M</t>
         </is>
       </c>
-      <c r="H14" s="4" t="n"/>
+      <c r="H14" s="6" t="n">
+        <v>0.05</v>
+      </c>
       <c r="I14" s="4" t="n"/>
-      <c r="J14" s="6" t="n">
+      <c r="J14" s="7" t="n">
         <v>1.9</v>
       </c>
       <c r="K14" s="4" t="inlineStr">
@@ -1068,9 +1094,11 @@
           <t>PC</t>
         </is>
       </c>
-      <c r="H15" s="4" t="n"/>
+      <c r="H15" s="6" t="n">
+        <v>0.01</v>
+      </c>
       <c r="I15" s="4" t="n"/>
-      <c r="J15" s="6" t="n">
+      <c r="J15" s="7" t="n">
         <v>0.08</v>
       </c>
       <c r="K15" s="4" t="inlineStr">
@@ -1085,139 +1113,148 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>Q35 celkem (faktura 810678974)</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>143952-0-0-00-FRP</t>
         </is>
       </c>
-      <c r="C16" s="7" t="n"/>
-      <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
-      <c r="F16" s="7">
+      <c r="C16" s="8" t="n"/>
+      <c r="D16" s="8" t="n"/>
+      <c r="E16" s="8" t="n"/>
+      <c r="F16" s="8">
         <f>SUM(F12:F15)</f>
         <v>34</v>
       </c>
-      <c r="G16" s="7" t="n"/>
-      <c r="H16" s="8" t="n">
+      <c r="G16" s="8" t="n"/>
+      <c r="H16" s="9">
+        <f>SUM(H12:H15)</f>
         <v>1.5</v>
       </c>
-      <c r="I16" s="8" t="n">
+      <c r="I16" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="J16" s="9">
+      <c r="J16" s="11">
         <f>SUM(J12:J15)</f>
         <v>56.28</v>
       </c>
-      <c r="K16" s="7" t="n"/>
-      <c r="L16" s="7" t="n"/>
+      <c r="K16" s="8" t="n"/>
+      <c r="L16" s="8" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>Zásilka celkem</t>
         </is>
       </c>
-      <c r="B17" s="10" t="n"/>
-      <c r="C17" s="10" t="n"/>
-      <c r="D17" s="10" t="n"/>
-      <c r="E17" s="10" t="n"/>
-      <c r="F17" s="10" t="n"/>
-      <c r="G17" s="10" t="n"/>
-      <c r="H17" s="11">
+      <c r="B17" s="12" t="n"/>
+      <c r="C17" s="12" t="n"/>
+      <c r="D17" s="12" t="n"/>
+      <c r="E17" s="12" t="n"/>
+      <c r="F17" s="12" t="n"/>
+      <c r="G17" s="12" t="n"/>
+      <c r="H17" s="13">
         <f>H11+H16</f>
         <v>4</v>
       </c>
-      <c r="I17" s="11">
+      <c r="I17" s="14">
         <f>I11+I16</f>
         <v>5</v>
       </c>
-      <c r="J17" s="12">
+      <c r="J17" s="15">
         <f>J11+J16</f>
         <v>1105.71</v>
       </c>
-      <c r="K17" s="10" t="n"/>
-      <c r="L17" s="10" t="n"/>
+      <c r="K17" s="12" t="n"/>
+      <c r="L17" s="12" t="n"/>
     </row>
     <row r="19" ht="15" customHeight="1">
-      <c r="A19" s="13" t="inlineStr">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>POZNÁMKY:</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="13" t="inlineStr">
-        <is>
-          <t>• REFERENCE: Oba balíčky (P35 i Q35) mají v e-mailu STEJNOU referenci 143952-0-0-00-FRP — dělení podle reference se tedy kryje s dělením podle balíčků. Číslo objednávky 4501839901 (pro interní účtování Hitachi) je uvedeno v hlavičce.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="14" t="inlineStr">
+    <row r="20" ht="42" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>⚠ ČISTÉ HMOTNOSTI = ODHAD: Faktury uvádějí u všech položek 'Net Weight 0', proto jsou čisté hmotnosti na řádcích POUZE PŘIBLIŽNÝ ODHAD (kurzívou) — rozděleny podle typu zboží (spojovací materiál = gramy; sada štítků, kryty a držák = většina hmotnosti) tak, aby součet za balíček odpovídal dokladům: P35 NW 2,5 kg, Q35 NW 1,5 kg. Pro přesné hodnoty je třeba vyžádat hmotnosti položek od Hitachi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="42" customHeight="1">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>• REFERENCE: Oba balíčky (P35 i Q35) mají v e-mailu STEJNOU referenci 143952-0-0-00-FRP — dělení podle reference se kryje s dělením podle balíčků. Číslo objednávky 4501839901 (pro interní účtování Hitachi) je uvedeno v hlavičce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>⚠ PREFERENČNÍ VĚTA: V dokladech (faktury 810678973/810678974, dodací listy) NENÍ uvedena žádná preferenční věta o původu. Zboží nemá deklarován preferenční původ.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="14" t="inlineStr">
-        <is>
-          <t>⚠ HMOTNOSTI: Faktury uvádějí u všech položek 'Net Weight 0' — čistá/hrubá hmotnost na úrovni jednotlivých HS kódů NENÍ v podkladech k dispozici. Uvedeny jsou pouze hmotnosti za balíček (P35: NW 2,5 kg / GW 3 kg; Q35: NW 1,5 kg / GW 2 kg — zdroj: e-mail Hitachi + dodací listy). Sloupce ponechány dle pravidel.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="15" t="inlineStr">
+    <row r="23" ht="15" customHeight="1">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
+          <t>• Hrubá hmotnost je k dispozici pouze za balíček (P35: 3 kg, Q35: 2 kg — dodací listy), na řádcích proto není rozepsána.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="18" t="inlineStr">
         <is>
           <t>• Hodnoty řádků odpovídají fakturám: P35 = 1 049,43 EUR (faktura 810678973), Q35 = 56,28 EUR (faktura 810678974). Kontrolní součty sedí na fakturované částky.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="15" t="inlineStr">
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="18" t="inlineStr">
         <is>
           <t>• CBAM: kódy 7318/7326 (železo/ocel) jsou v příloze I nařízení CBAM — relevantní při dovozu do EU; tato zásilka je vývoz z EU, CBAM se na ni tedy přímo nevztahuje.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="15" t="inlineStr">
+    <row r="26" ht="42" customHeight="1">
+      <c r="A26" s="18" t="inlineStr">
         <is>
           <t>• Antidumping: samosvorné matice (73181650) původem z Číny podléhají při dovozu do EU antidumpingovému clu na spojovací materiál (nař. 2022/191) — pro tento vývoz bez přímého dopadu, uvedeno pro úplnost.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1">
-      <c r="A26" s="15" t="inlineStr">
+    <row r="27" ht="15" customHeight="1">
+      <c r="A27" s="18" t="inlineStr">
         <is>
           <t>• Popisy (CZ) dodány zákazníkem e-mailem (Iva Kolertová, Hitachi Energy, 20.07.2026).</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="15" customHeight="1">
-      <c r="A27" s="15" t="inlineStr">
+    <row r="28" ht="15" customHeight="1">
+      <c r="A28" s="18" t="inlineStr">
         <is>
           <t>• Bez obchodní slevy — žádná sleva na fakturách uvedena není.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1">
-      <c r="A28" s="15" t="inlineStr">
+    <row r="29" ht="15" customHeight="1">
+      <c r="A29" s="18" t="inlineStr">
         <is>
           <t>• Incoterm CPT Eemshaven (dle pravidel neuveden jako sloupec). Projekt: offshore Nordsee 2 / Godewind.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="A20:L20"/>
     <mergeCell ref="A24:L24"/>
     <mergeCell ref="A26:L26"/>
+    <mergeCell ref="A29:L29"/>
     <mergeCell ref="A25:L25"/>
     <mergeCell ref="A19:L19"/>
     <mergeCell ref="A28:L28"/>

</xml_diff>

<commit_message>
Add invoice and delivery note numbers per HS row; remove CBAM column
CBAM dropped per user — this is an EU export, CBAM is not handled here.
Each HS code row now carries its invoice number (P35: 810678973,
Q35: 810678974) and delivery note number (P35: 0923629561,
Q35: 0923629583).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P7dj9YaDaJdQUHninPzxpV
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Hitachi_143952.xlsx
+++ b/output/HS_Code_Summary_Hitachi_143952.xlsx
@@ -498,21 +498,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:M28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="6" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="38" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="38" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -542,50 +543,55 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
+          <t>Faktura č.</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Dodací list č.</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
           <t>HS kód</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Popis (CZ)</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Země původu</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Množství</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>MJ</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Čistá hmotnost (kg) — ODHAD</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Hrubá hmotnost (kg)</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>Celní hodnota (EUR)</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>CBAM</t>
-        </is>
-      </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>Antidumping</t>
         </is>
@@ -604,40 +610,45 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
+          <t>810678973</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>0923629561</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
           <t>73269098</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>Ostatní výrobky ze železa nebo oceli, které nejsou nikde jinde specifikovány</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>CZ</t>
         </is>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="H5" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="H5" s="6" t="n">
+      <c r="J5" s="6" t="n">
         <v>0.5</v>
       </c>
-      <c r="I5" s="4" t="n"/>
-      <c r="J5" s="7" t="n">
+      <c r="K5" s="4" t="n"/>
+      <c r="L5" s="7" t="n">
         <v>10.89</v>
       </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>Ano (příloha I CBAM)</t>
-        </is>
-      </c>
-      <c r="L5" s="5" t="inlineStr"/>
+      <c r="M5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -652,40 +663,45 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
+          <t>810678973</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>0923629561</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
           <t>73181650</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>Samosvorné matice</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="H6" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="H6" s="6" t="n">
+      <c r="J6" s="6" t="n">
         <v>0.02</v>
       </c>
-      <c r="I6" s="4" t="n"/>
-      <c r="J6" s="7" t="n">
+      <c r="K6" s="4" t="n"/>
+      <c r="L6" s="7" t="n">
         <v>0.52</v>
       </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>Ano (příloha I CBAM)</t>
-        </is>
-      </c>
-      <c r="L6" s="5" t="inlineStr">
+      <c r="M6" s="5" t="inlineStr">
         <is>
           <t>Spojovací materiál ze železa/oceli původem CN — dovoz do EU podléhá antidumpingu (nař. 2022/191)</t>
         </is>
@@ -704,40 +720,45 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
+          <t>810678973</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>0923629561</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
           <t>74153300</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>Šrouby, vruty, svorníky (maticové šrouby) a matice z mědi, případně ze železa nebo oceli s měděnou hlavou</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="H7" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="H7" s="6" t="n">
+      <c r="J7" s="6" t="n">
         <v>0.03</v>
       </c>
-      <c r="I7" s="4" t="n"/>
-      <c r="J7" s="7" t="n">
+      <c r="K7" s="4" t="n"/>
+      <c r="L7" s="7" t="n">
         <v>0.35</v>
       </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t>Ne</t>
-        </is>
-      </c>
-      <c r="L7" s="5" t="inlineStr"/>
+      <c r="M7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -752,40 +773,45 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
+          <t>810678973</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>0923629561</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
           <t>39269097</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>Ostatní výrobky z plastů, které nejsou jinde specifikovány</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>CZ</t>
         </is>
       </c>
-      <c r="F8" s="4" t="n">
+      <c r="H8" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="H8" s="6" t="n">
+      <c r="J8" s="6" t="n">
         <v>1.8</v>
       </c>
-      <c r="I8" s="4" t="n"/>
-      <c r="J8" s="7" t="n">
+      <c r="K8" s="4" t="n"/>
+      <c r="L8" s="7" t="n">
         <v>1002.9</v>
       </c>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>Ne</t>
-        </is>
-      </c>
-      <c r="L8" s="5" t="inlineStr"/>
+      <c r="M8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -800,40 +826,45 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
+          <t>810678973</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>0923629561</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
           <t>85381000</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>Tabule, panely, ovládací stoly, pulty, skříně a jiné základny pro elektrické řízení nebo rozvod elektřiny, které nejsou vybaveny příslušnými přístroji</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>CZ</t>
         </is>
       </c>
-      <c r="F9" s="4" t="n">
+      <c r="H9" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="H9" s="6" t="n">
+      <c r="J9" s="6" t="n">
         <v>0.1</v>
       </c>
-      <c r="I9" s="4" t="n"/>
-      <c r="J9" s="7" t="n">
+      <c r="K9" s="4" t="n"/>
+      <c r="L9" s="7" t="n">
         <v>32.87</v>
       </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>Ne</t>
-        </is>
-      </c>
-      <c r="L9" s="5" t="inlineStr"/>
+      <c r="M9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -848,45 +879,50 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
+          <t>810678973</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>0923629561</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
           <t>40169300</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>Plochá těsnění, podložky a jiná těsnění</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>AT</t>
         </is>
       </c>
-      <c r="F10" s="4" t="n">
+      <c r="H10" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="H10" s="6" t="n">
+      <c r="J10" s="6" t="n">
         <v>0.05</v>
       </c>
-      <c r="I10" s="4" t="n"/>
-      <c r="J10" s="7" t="n">
+      <c r="K10" s="4" t="n"/>
+      <c r="L10" s="7" t="n">
         <v>1.9</v>
       </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>Ne</t>
-        </is>
-      </c>
-      <c r="L10" s="5" t="inlineStr"/>
+      <c r="M10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>P35 celkem (faktura 810678973)</t>
+          <t>P35 celkem</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
@@ -894,27 +930,36 @@
           <t>143952-0-0-00-FRP</t>
         </is>
       </c>
-      <c r="C11" s="8" t="n"/>
-      <c r="D11" s="8" t="n"/>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>810678973</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>0923629561</t>
+        </is>
+      </c>
       <c r="E11" s="8" t="n"/>
-      <c r="F11" s="8">
-        <f>SUM(F5:F10)</f>
+      <c r="F11" s="8" t="n"/>
+      <c r="G11" s="8" t="n"/>
+      <c r="H11" s="8">
+        <f>SUM(H5:H10)</f>
         <v>37</v>
       </c>
-      <c r="G11" s="8" t="n"/>
-      <c r="H11" s="9">
-        <f>SUM(H5:H10)</f>
+      <c r="I11" s="8" t="n"/>
+      <c r="J11" s="9">
+        <f>SUM(J5:J10)</f>
         <v>2.5</v>
       </c>
-      <c r="I11" s="10" t="n">
+      <c r="K11" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="J11" s="11">
-        <f>SUM(J5:J10)</f>
+      <c r="L11" s="11">
+        <f>SUM(L5:L10)</f>
         <v>1049.43</v>
       </c>
-      <c r="K11" s="8" t="n"/>
-      <c r="L11" s="8" t="n"/>
+      <c r="M11" s="8" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -929,40 +974,45 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
+          <t>810678974</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>0923629583</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
           <t>85381000</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>Tabule, panely, ovládací stoly, pulty, skříně a jiné základny pro elektrické řízení nebo rozvod elektřiny, které nejsou vybaveny příslušnými přístroji</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>CZ</t>
         </is>
       </c>
-      <c r="F12" s="4" t="n">
+      <c r="H12" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="H12" s="6" t="n">
+      <c r="J12" s="6" t="n">
         <v>1.4</v>
       </c>
-      <c r="I12" s="4" t="n"/>
-      <c r="J12" s="7" t="n">
+      <c r="K12" s="4" t="n"/>
+      <c r="L12" s="7" t="n">
         <v>53.66</v>
       </c>
-      <c r="K12" s="4" t="inlineStr">
-        <is>
-          <t>Ne</t>
-        </is>
-      </c>
-      <c r="L12" s="5" t="inlineStr"/>
+      <c r="M12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -977,40 +1027,45 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
+          <t>810678974</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>0923629583</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
           <t>74153300</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>Šrouby, vruty, svorníky (maticové šrouby) a matice z mědi, případně ze železa nebo oceli s měděnou hlavou</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="F13" s="4" t="n">
+      <c r="H13" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="H13" s="6" t="n">
+      <c r="J13" s="6" t="n">
         <v>0.04</v>
       </c>
-      <c r="I13" s="4" t="n"/>
-      <c r="J13" s="7" t="n">
+      <c r="K13" s="4" t="n"/>
+      <c r="L13" s="7" t="n">
         <v>0.64</v>
       </c>
-      <c r="K13" s="4" t="inlineStr">
-        <is>
-          <t>Ne</t>
-        </is>
-      </c>
-      <c r="L13" s="5" t="inlineStr"/>
+      <c r="M13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1025,40 +1080,45 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
+          <t>810678974</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>0923629583</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
           <t>40169300</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>Plochá těsnění, podložky a jiná těsnění</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>AT</t>
         </is>
       </c>
-      <c r="F14" s="4" t="n">
+      <c r="H14" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="H14" s="6" t="n">
+      <c r="J14" s="6" t="n">
         <v>0.05</v>
       </c>
-      <c r="I14" s="4" t="n"/>
-      <c r="J14" s="7" t="n">
+      <c r="K14" s="4" t="n"/>
+      <c r="L14" s="7" t="n">
         <v>1.9</v>
       </c>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t>Ne</t>
-        </is>
-      </c>
-      <c r="L14" s="5" t="inlineStr"/>
+      <c r="M14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1073,40 +1133,45 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
+          <t>810678974</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>0923629583</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
           <t>73181650</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>Samosvorné matice</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="F15" s="4" t="n">
+      <c r="H15" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="H15" s="6" t="n">
+      <c r="J15" s="6" t="n">
         <v>0.01</v>
       </c>
-      <c r="I15" s="4" t="n"/>
-      <c r="J15" s="7" t="n">
+      <c r="K15" s="4" t="n"/>
+      <c r="L15" s="7" t="n">
         <v>0.08</v>
       </c>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t>Ano (příloha I CBAM)</t>
-        </is>
-      </c>
-      <c r="L15" s="5" t="inlineStr">
+      <c r="M15" s="5" t="inlineStr">
         <is>
           <t>Spojovací materiál ze železa/oceli původem CN — dovoz do EU podléhá antidumpingu (nař. 2022/191)</t>
         </is>
@@ -1115,7 +1180,7 @@
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>Q35 celkem (faktura 810678974)</t>
+          <t>Q35 celkem</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
@@ -1123,27 +1188,36 @@
           <t>143952-0-0-00-FRP</t>
         </is>
       </c>
-      <c r="C16" s="8" t="n"/>
-      <c r="D16" s="8" t="n"/>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>810678974</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>0923629583</t>
+        </is>
+      </c>
       <c r="E16" s="8" t="n"/>
-      <c r="F16" s="8">
-        <f>SUM(F12:F15)</f>
+      <c r="F16" s="8" t="n"/>
+      <c r="G16" s="8" t="n"/>
+      <c r="H16" s="8">
+        <f>SUM(H12:H15)</f>
         <v>34</v>
       </c>
-      <c r="G16" s="8" t="n"/>
-      <c r="H16" s="9">
-        <f>SUM(H12:H15)</f>
+      <c r="I16" s="8" t="n"/>
+      <c r="J16" s="9">
+        <f>SUM(J12:J15)</f>
         <v>1.5</v>
       </c>
-      <c r="I16" s="10" t="n">
+      <c r="K16" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="J16" s="11">
-        <f>SUM(J12:J15)</f>
+      <c r="L16" s="11">
+        <f>SUM(L12:L15)</f>
         <v>56.28</v>
       </c>
-      <c r="K16" s="8" t="n"/>
-      <c r="L16" s="8" t="n"/>
+      <c r="M16" s="8" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
@@ -1157,20 +1231,21 @@
       <c r="E17" s="12" t="n"/>
       <c r="F17" s="12" t="n"/>
       <c r="G17" s="12" t="n"/>
-      <c r="H17" s="13">
-        <f>H11+H16</f>
+      <c r="H17" s="12" t="n"/>
+      <c r="I17" s="12" t="n"/>
+      <c r="J17" s="13">
+        <f>J11+J16</f>
         <v>4</v>
       </c>
-      <c r="I17" s="14">
-        <f>I11+I16</f>
+      <c r="K17" s="14">
+        <f>K11+K16</f>
         <v>5</v>
       </c>
-      <c r="J17" s="15">
-        <f>J11+J16</f>
+      <c r="L17" s="15">
+        <f>L11+L16</f>
         <v>1105.71</v>
       </c>
-      <c r="K17" s="12" t="n"/>
-      <c r="L17" s="12" t="n"/>
+      <c r="M17" s="12" t="n"/>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="16" t="inlineStr">
@@ -1182,14 +1257,14 @@
     <row r="20" ht="42" customHeight="1">
       <c r="A20" s="17" t="inlineStr">
         <is>
-          <t>⚠ ČISTÉ HMOTNOSTI = ODHAD: Faktury uvádějí u všech položek 'Net Weight 0', proto jsou čisté hmotnosti na řádcích POUZE PŘIBLIŽNÝ ODHAD (kurzívou) — rozděleny podle typu zboží (spojovací materiál = gramy; sada štítků, kryty a držák = většina hmotnosti) tak, aby součet za balíček odpovídal dokladům: P35 NW 2,5 kg, Q35 NW 1,5 kg. Pro přesné hodnoty je třeba vyžádat hmotnosti položek od Hitachi.</t>
+          <t>⚠ ČISTÉ HMOTNOSTI = ODHAD: Faktury uvádějí u všech položek 'Net Weight 0', proto jsou čisté hmotnosti na řádcích POUZE PŘIBLIŽNÝ ODHAD (kurzívou) — rozděleny podle typu zboží tak, aby součet za balíček odpovídal dokladům: P35 NW 2,5 kg, Q35 NW 1,5 kg. Pro přesné hodnoty je třeba vyžádat hmotnosti položek od Hitachi.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1">
       <c r="A21" s="16" t="inlineStr">
         <is>
-          <t>• REFERENCE: Oba balíčky (P35 i Q35) mají v e-mailu STEJNOU referenci 143952-0-0-00-FRP — dělení podle reference se kryje s dělením podle balíčků. Číslo objednávky 4501839901 (pro interní účtování Hitachi) je uvedeno v hlavičce.</t>
+          <t>• DOKLADY: P35 = faktura 810678973 + dodací list 0923629561; Q35 = faktura 810678974 + dodací list 0923629583. Oba balíčky mají v e-mailu stejnou referenci 143952-0-0-00-FRP; číslo objednávky 4501839901 v hlavičce.</t>
         </is>
       </c>
     </row>
@@ -1207,61 +1282,53 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="30" customHeight="1">
+    <row r="24" ht="15" customHeight="1">
       <c r="A24" s="18" t="inlineStr">
         <is>
-          <t>• Hodnoty řádků odpovídají fakturám: P35 = 1 049,43 EUR (faktura 810678973), Q35 = 56,28 EUR (faktura 810678974). Kontrolní součty sedí na fakturované částky.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="30" customHeight="1">
+          <t>• Hodnoty řádků odpovídají fakturám: P35 = 1 049,43 EUR, Q35 = 56,28 EUR. Kontrolní součty sedí na fakturované částky.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="42" customHeight="1">
       <c r="A25" s="18" t="inlineStr">
         <is>
-          <t>• CBAM: kódy 7318/7326 (železo/ocel) jsou v příloze I nařízení CBAM — relevantní při dovozu do EU; tato zásilka je vývoz z EU, CBAM se na ni tedy přímo nevztahuje.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="42" customHeight="1">
+          <t>• Antidumping: samosvorné matice (73181650) původem z Číny podléhají při dovozu do EU antidumpingovému clu na spojovací materiál (nař. 2022/191) — pro tento vývoz bez přímého dopadu, uvedeno pro úplnost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="15" customHeight="1">
       <c r="A26" s="18" t="inlineStr">
         <is>
-          <t>• Antidumping: samosvorné matice (73181650) původem z Číny podléhají při dovozu do EU antidumpingovému clu na spojovací materiál (nař. 2022/191) — pro tento vývoz bez přímého dopadu, uvedeno pro úplnost.</t>
+          <t>• Popisy (CZ) dodány zákazníkem e-mailem (Iva Kolertová, Hitachi Energy, 20.07.2026).</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="18" t="inlineStr">
         <is>
-          <t>• Popisy (CZ) dodány zákazníkem e-mailem (Iva Kolertová, Hitachi Energy, 20.07.2026).</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="15" customHeight="1">
+          <t>• Bez obchodní slevy — žádná sleva na fakturách uvedena není.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
       <c r="A28" s="18" t="inlineStr">
         <is>
-          <t>• Bez obchodní slevy — žádná sleva na fakturách uvedena není.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="15" customHeight="1">
-      <c r="A29" s="18" t="inlineStr">
-        <is>
-          <t>• Incoterm CPT Eemshaven (dle pravidel neuveden jako sloupec). Projekt: offshore Nordsee 2 / Godewind.</t>
+          <t>• Incoterm CPT Eemshaven (dle pravidel neuveden jako sloupec). Projekt: offshore Nordsee 2 / Godewind. Vývoz z EU — CBAM se neřeší.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="A20:L20"/>
-    <mergeCell ref="A24:L24"/>
-    <mergeCell ref="A26:L26"/>
-    <mergeCell ref="A29:L29"/>
-    <mergeCell ref="A25:L25"/>
-    <mergeCell ref="A19:L19"/>
-    <mergeCell ref="A28:L28"/>
-    <mergeCell ref="A23:L23"/>
-    <mergeCell ref="A22:L22"/>
-    <mergeCell ref="A27:L27"/>
-    <mergeCell ref="A21:L21"/>
+  <mergeCells count="10">
+    <mergeCell ref="A19:M19"/>
+    <mergeCell ref="A23:M23"/>
+    <mergeCell ref="A27:M27"/>
+    <mergeCell ref="A22:M22"/>
+    <mergeCell ref="A26:M26"/>
+    <mergeCell ref="A21:M21"/>
+    <mergeCell ref="A25:M25"/>
+    <mergeCell ref="A20:M20"/>
+    <mergeCell ref="A24:M24"/>
+    <mergeCell ref="A28:M28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>